<commit_message>
fix(impostos): ajuste da apuracao tributaria e parcelamentos conforme planilha atualizada
</commit_message>
<xml_diff>
--- a/parcelamentos_local.xlsx
+++ b/parcelamentos_local.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\10.121.21.252\controladoria\Vitor\TRIBUTARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F3F6A7E3-F71E-4C60-AB83-7CCCE56916EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71E595A2-57D5-4FA1-BA2F-B8E781543CB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="804" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="804" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="PARCELAMENTOS" sheetId="1" r:id="rId1"/>
-    <sheet name="PARCELAMENTO 06062024" sheetId="4" r:id="rId2"/>
-    <sheet name="PARCELAMENTO 05122024" sheetId="2" r:id="rId3"/>
-    <sheet name="PARCELAMENTO 06062025" sheetId="10" r:id="rId4"/>
-    <sheet name="PARCELAMENTO 25112025 " sheetId="13" r:id="rId5"/>
-    <sheet name="PARCELAMENTO SC" sheetId="12" r:id="rId6"/>
-    <sheet name="IMPOSTOS NÃO PARCELADOS" sheetId="9" r:id="rId7"/>
-    <sheet name="ACOMPANHAMENTO MENSAL" sheetId="11" r:id="rId8"/>
+    <sheet name="SALDO CREDOR INSS" sheetId="14" r:id="rId1"/>
+    <sheet name="PARCELAMENTOS" sheetId="1" r:id="rId2"/>
+    <sheet name="PARCELAMENTO 06062024" sheetId="4" r:id="rId3"/>
+    <sheet name="PARCELAMENTO 05122024" sheetId="2" r:id="rId4"/>
+    <sheet name="PARCELAMENTO 06062025" sheetId="10" r:id="rId5"/>
+    <sheet name="PARCELAMENTO 25112025 " sheetId="13" r:id="rId6"/>
+    <sheet name="PARCELAMENTO SC" sheetId="12" r:id="rId7"/>
+    <sheet name="IMPOSTOS NÃO PARCELADOS" sheetId="9" r:id="rId8"/>
+    <sheet name="ACOMPANHAMENTO MENSAL" sheetId="11" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -104,7 +105,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="111">
   <si>
     <t>TAURA AGRONEGOCIOS - IMPOSTOS EM ABERTO - NÃO PARCELADOS NA RECEITA FEDERAL</t>
   </si>
@@ -423,6 +424,21 @@
   <si>
     <t>Parcelamento 25/11/2025</t>
   </si>
+  <si>
+    <t>SALDO CREDOR INSS - JLE</t>
+  </si>
+  <si>
+    <t>COMPETÊNCIA</t>
+  </si>
+  <si>
+    <t>RETENÇÃO NF</t>
+  </si>
+  <si>
+    <t>UTILIZADO FOLHA</t>
+  </si>
+  <si>
+    <t>SALDO</t>
+  </si>
 </sst>
 </file>
 
@@ -433,7 +449,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-&quot;R$&quot;* #,##0.00_-;\-&quot;R$&quot;* #,##0.00_-;_-&quot;R$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -562,6 +578,34 @@
       <b/>
       <sz val="9"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -956,7 +1000,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="140">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1156,6 +1200,18 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="43" fontId="3" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1172,18 +1228,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -1203,6 +1247,61 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="4" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="18" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="5" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="4" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="39" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="20" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="21" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="19" fillId="5" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="19" fillId="5" borderId="11" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="19" fillId="5" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="19" fillId="5" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="39" fontId="19" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="39" fontId="19" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="21" fillId="8" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -4802,6 +4901,538 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A737B4A5-C227-4B65-8FEE-4CA1A32A001E}">
+  <dimension ref="A1:G61"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="5.33203125" style="114" customWidth="1"/>
+    <col min="2" max="2" width="11.77734375" style="114" customWidth="1"/>
+    <col min="3" max="3" width="18" style="114" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.77734375" style="114" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" style="114" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3.6640625" style="114" customWidth="1"/>
+    <col min="7" max="7" width="15.88671875" style="114" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="3.88671875" style="114" customWidth="1"/>
+    <col min="9" max="9" width="12.6640625" style="114" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.88671875" style="114" customWidth="1"/>
+    <col min="11" max="11" width="2.5546875" style="114" customWidth="1"/>
+    <col min="12" max="13" width="15.44140625" style="114" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="13.88671875" style="114" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.88671875" style="114" customWidth="1"/>
+    <col min="17" max="17" width="15.44140625" style="114" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.6640625" style="114" bestFit="1" customWidth="1"/>
+    <col min="19" max="16384" width="8.88671875" style="114"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="18.75" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="113"/>
+      <c r="B1" s="113"/>
+      <c r="C1" s="113"/>
+      <c r="D1" s="113"/>
+      <c r="E1" s="113"/>
+      <c r="F1" s="113"/>
+      <c r="G1" s="113"/>
+    </row>
+    <row r="2" spans="1:7" s="115" customFormat="1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="116"/>
+      <c r="C2" s="116"/>
+      <c r="D2" s="116"/>
+      <c r="E2" s="116"/>
+      <c r="F2" s="116"/>
+      <c r="G2" s="116"/>
+    </row>
+    <row r="3" spans="1:7" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="117"/>
+      <c r="C3" s="117"/>
+      <c r="D3" s="117"/>
+      <c r="E3" s="117"/>
+      <c r="F3" s="117"/>
+      <c r="G3" s="117"/>
+    </row>
+    <row r="4" spans="1:7" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="117"/>
+      <c r="C4" s="117"/>
+      <c r="D4" s="117"/>
+      <c r="E4" s="117"/>
+      <c r="F4" s="117"/>
+      <c r="G4" s="117"/>
+    </row>
+    <row r="5" spans="1:7" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="117"/>
+      <c r="C5" s="117"/>
+      <c r="D5" s="117"/>
+      <c r="E5" s="117"/>
+      <c r="F5" s="117"/>
+      <c r="G5" s="117"/>
+    </row>
+    <row r="6" spans="1:7" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="118"/>
+      <c r="B6" s="119"/>
+      <c r="C6" s="119"/>
+      <c r="D6" s="119"/>
+      <c r="E6" s="119"/>
+      <c r="F6" s="119"/>
+      <c r="G6" s="119"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="113"/>
+      <c r="B8" s="130" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" s="130"/>
+      <c r="D8" s="120"/>
+      <c r="E8" s="120"/>
+      <c r="F8" s="120"/>
+      <c r="G8" s="120"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="113"/>
+      <c r="B9" s="113"/>
+      <c r="C9" s="113"/>
+      <c r="D9" s="121"/>
+      <c r="E9" s="121"/>
+    </row>
+    <row r="10" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="122"/>
+      <c r="B10" s="131" t="s">
+        <v>107</v>
+      </c>
+      <c r="C10" s="131" t="s">
+        <v>108</v>
+      </c>
+      <c r="D10" s="131" t="s">
+        <v>109</v>
+      </c>
+      <c r="E10" s="131" t="s">
+        <v>110</v>
+      </c>
+      <c r="F10" s="123"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="124"/>
+      <c r="B11" s="132">
+        <v>46113</v>
+      </c>
+      <c r="C11" s="133">
+        <v>120627.34</v>
+      </c>
+      <c r="D11" s="134">
+        <v>102779.58</v>
+      </c>
+      <c r="E11" s="135">
+        <f>C11-D11</f>
+        <v>17847.759999999995</v>
+      </c>
+      <c r="F11" s="125"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="124"/>
+      <c r="B12" s="132">
+        <v>46143</v>
+      </c>
+      <c r="C12" s="133">
+        <v>126667.52</v>
+      </c>
+      <c r="D12" s="134">
+        <v>103847.05</v>
+      </c>
+      <c r="E12" s="135">
+        <f t="shared" ref="E12:E19" si="0">C12-D12</f>
+        <v>22820.47</v>
+      </c>
+      <c r="F12" s="126"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="124"/>
+      <c r="B13" s="132">
+        <v>46174</v>
+      </c>
+      <c r="C13" s="133">
+        <v>152096.76</v>
+      </c>
+      <c r="D13" s="134">
+        <v>95919.98</v>
+      </c>
+      <c r="E13" s="135">
+        <f t="shared" si="0"/>
+        <v>56176.780000000013</v>
+      </c>
+      <c r="F13" s="126"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="124"/>
+      <c r="B14" s="132">
+        <v>46204</v>
+      </c>
+      <c r="C14" s="133">
+        <v>135916.62</v>
+      </c>
+      <c r="D14" s="134">
+        <v>97086.87</v>
+      </c>
+      <c r="E14" s="135">
+        <f t="shared" si="0"/>
+        <v>38829.75</v>
+      </c>
+      <c r="F14" s="126"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="127"/>
+      <c r="B15" s="132">
+        <v>46235</v>
+      </c>
+      <c r="C15" s="136">
+        <v>124463.52</v>
+      </c>
+      <c r="D15" s="136">
+        <v>107769.34</v>
+      </c>
+      <c r="E15" s="135">
+        <f t="shared" si="0"/>
+        <v>16694.180000000008</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="127"/>
+      <c r="B16" s="132">
+        <v>46266</v>
+      </c>
+      <c r="C16" s="137"/>
+      <c r="D16" s="137"/>
+      <c r="E16" s="135">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="129"/>
+      <c r="B17" s="132">
+        <v>46296</v>
+      </c>
+      <c r="C17" s="137"/>
+      <c r="D17" s="137"/>
+      <c r="E17" s="135">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="127"/>
+      <c r="B18" s="132">
+        <v>46327</v>
+      </c>
+      <c r="C18" s="137"/>
+      <c r="D18" s="137"/>
+      <c r="E18" s="135">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="127"/>
+      <c r="B19" s="132">
+        <v>46357</v>
+      </c>
+      <c r="C19" s="137"/>
+      <c r="D19" s="137"/>
+      <c r="E19" s="135">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="127"/>
+      <c r="B20" s="138"/>
+      <c r="C20" s="138"/>
+      <c r="D20" s="138"/>
+      <c r="E20" s="139">
+        <f>SUM(E11:E19)</f>
+        <v>152368.94</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="127"/>
+      <c r="B21" s="128"/>
+      <c r="C21" s="128"/>
+      <c r="D21" s="128"/>
+      <c r="E21" s="128"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="127"/>
+      <c r="B22" s="128"/>
+      <c r="C22" s="128"/>
+      <c r="D22" s="128"/>
+      <c r="E22" s="128"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="127"/>
+      <c r="B23" s="128"/>
+      <c r="C23" s="128"/>
+      <c r="D23" s="128"/>
+      <c r="E23" s="128"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="127"/>
+      <c r="B24" s="128"/>
+      <c r="C24" s="128"/>
+      <c r="D24" s="128"/>
+      <c r="E24" s="128"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="127"/>
+      <c r="B25" s="128"/>
+      <c r="C25" s="128"/>
+      <c r="D25" s="128"/>
+      <c r="E25" s="128"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="127"/>
+      <c r="B26" s="128"/>
+      <c r="C26" s="128"/>
+      <c r="D26" s="128"/>
+      <c r="E26" s="128"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="127"/>
+      <c r="B27" s="128"/>
+      <c r="C27" s="128"/>
+      <c r="D27" s="128"/>
+      <c r="E27" s="128"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="127"/>
+      <c r="B28" s="128"/>
+      <c r="C28" s="128"/>
+      <c r="D28" s="128"/>
+      <c r="E28" s="128"/>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" s="127"/>
+      <c r="B29" s="128"/>
+      <c r="C29" s="128"/>
+      <c r="D29" s="128"/>
+      <c r="E29" s="128"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" s="127"/>
+      <c r="B30" s="128"/>
+      <c r="C30" s="128"/>
+      <c r="D30" s="128"/>
+      <c r="E30" s="128"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" s="127"/>
+      <c r="B31" s="128"/>
+      <c r="C31" s="128"/>
+      <c r="D31" s="128"/>
+      <c r="E31" s="128"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" s="127"/>
+      <c r="B32" s="128"/>
+      <c r="C32" s="128"/>
+      <c r="D32" s="128"/>
+      <c r="E32" s="128"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" s="127"/>
+      <c r="B33" s="128"/>
+      <c r="C33" s="128"/>
+      <c r="D33" s="128"/>
+      <c r="E33" s="128"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34" s="127"/>
+      <c r="B34" s="128"/>
+      <c r="C34" s="128"/>
+      <c r="D34" s="128"/>
+      <c r="E34" s="128"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" s="127"/>
+      <c r="B35" s="128"/>
+      <c r="C35" s="128"/>
+      <c r="D35" s="128"/>
+      <c r="E35" s="128"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" s="127"/>
+      <c r="B36" s="128"/>
+      <c r="C36" s="128"/>
+      <c r="D36" s="128"/>
+      <c r="E36" s="128"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" s="127"/>
+      <c r="B37" s="128"/>
+      <c r="C37" s="128"/>
+      <c r="D37" s="128"/>
+      <c r="E37" s="128"/>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" s="127"/>
+      <c r="B38" s="128"/>
+      <c r="C38" s="128"/>
+      <c r="D38" s="128"/>
+      <c r="E38" s="128"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" s="127"/>
+      <c r="B39" s="128"/>
+      <c r="C39" s="128"/>
+      <c r="D39" s="128"/>
+      <c r="E39" s="128"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" s="127"/>
+      <c r="B40" s="128"/>
+      <c r="C40" s="128"/>
+      <c r="D40" s="128"/>
+      <c r="E40" s="128"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" s="127"/>
+      <c r="B41" s="128"/>
+      <c r="C41" s="128"/>
+      <c r="D41" s="128"/>
+      <c r="E41" s="128"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" s="127"/>
+      <c r="B42" s="128"/>
+      <c r="C42" s="128"/>
+      <c r="D42" s="128"/>
+      <c r="E42" s="128"/>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" s="127"/>
+      <c r="B43" s="128"/>
+      <c r="C43" s="128"/>
+      <c r="D43" s="128"/>
+      <c r="E43" s="128"/>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" s="127"/>
+      <c r="B44" s="128"/>
+      <c r="C44" s="128"/>
+      <c r="D44" s="128"/>
+      <c r="E44" s="128"/>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" s="127"/>
+      <c r="B45" s="128"/>
+      <c r="C45" s="128"/>
+      <c r="D45" s="128"/>
+      <c r="E45" s="128"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" s="127"/>
+      <c r="B46" s="128"/>
+      <c r="C46" s="128"/>
+      <c r="D46" s="128"/>
+      <c r="E46" s="128"/>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" s="127"/>
+      <c r="B47" s="128"/>
+      <c r="C47" s="128"/>
+      <c r="D47" s="128"/>
+      <c r="E47" s="128"/>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" s="127"/>
+      <c r="B48" s="128"/>
+      <c r="C48" s="128"/>
+      <c r="D48" s="128"/>
+      <c r="E48" s="128"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" s="127"/>
+      <c r="B49" s="128"/>
+      <c r="C49" s="128"/>
+      <c r="D49" s="128"/>
+      <c r="E49" s="128"/>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" s="127"/>
+      <c r="B50" s="128"/>
+      <c r="C50" s="128"/>
+      <c r="D50" s="128"/>
+      <c r="E50" s="128"/>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" s="127"/>
+      <c r="B51" s="128"/>
+      <c r="C51" s="128"/>
+      <c r="D51" s="128"/>
+      <c r="E51" s="128"/>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A52" s="127"/>
+      <c r="B52" s="128"/>
+      <c r="C52" s="128"/>
+      <c r="D52" s="128"/>
+      <c r="E52" s="128"/>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A53" s="127"/>
+      <c r="B53" s="128"/>
+      <c r="C53" s="128"/>
+      <c r="D53" s="128"/>
+      <c r="E53" s="128"/>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A54" s="127"/>
+      <c r="B54" s="128"/>
+      <c r="C54" s="128"/>
+      <c r="D54" s="128"/>
+      <c r="E54" s="128"/>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A55" s="127"/>
+      <c r="B55" s="128"/>
+      <c r="C55" s="128"/>
+      <c r="D55" s="128"/>
+      <c r="E55" s="128"/>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A56" s="127"/>
+      <c r="B56" s="128"/>
+      <c r="C56" s="128"/>
+      <c r="D56" s="128"/>
+      <c r="E56" s="128"/>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A57" s="127"/>
+      <c r="B57" s="128"/>
+      <c r="C57" s="128"/>
+      <c r="D57" s="128"/>
+      <c r="E57" s="128"/>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A58" s="127"/>
+      <c r="E58" s="128"/>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A59" s="127"/>
+      <c r="E59" s="128"/>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A60" s="127"/>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A61" s="127"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B8:C8"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G62"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4824,15 +5455,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18.75" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="101" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="98"/>
-      <c r="C1" s="98"/>
-      <c r="D1" s="98"/>
-      <c r="E1" s="98"/>
-      <c r="F1" s="98"/>
-      <c r="G1" s="99"/>
+      <c r="B1" s="102"/>
+      <c r="C1" s="102"/>
+      <c r="D1" s="102"/>
+      <c r="E1" s="102"/>
+      <c r="F1" s="102"/>
+      <c r="G1" s="103"/>
     </row>
     <row r="2" spans="1:7" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -4933,22 +5564,22 @@
     </row>
     <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="8" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="100" t="s">
+      <c r="A8" s="104" t="s">
         <v>78</v>
       </c>
-      <c r="B8" s="101"/>
-      <c r="C8" s="102"/>
+      <c r="B8" s="105"/>
+      <c r="C8" s="106"/>
       <c r="D8" s="12"/>
       <c r="E8" s="12"/>
       <c r="F8" s="12"/>
       <c r="G8" s="12"/>
     </row>
     <row r="9" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="100" t="s">
+      <c r="A9" s="104" t="s">
         <v>97</v>
       </c>
-      <c r="B9" s="101"/>
-      <c r="C9" s="102"/>
+      <c r="B9" s="105"/>
+      <c r="C9" s="106"/>
       <c r="D9" s="13"/>
       <c r="E9" s="13"/>
     </row>
@@ -5391,7 +6022,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B1:R85"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -5602,10 +6233,10 @@
         <f>M5-I6</f>
         <v>511198.30999999994</v>
       </c>
-      <c r="O6" s="103" t="s">
+      <c r="O6" s="97" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="103"/>
+      <c r="P6" s="97"/>
       <c r="Q6" s="82">
         <f>(Q4/O4)-1</f>
         <v>-0.43333314486548447</v>
@@ -5736,11 +6367,11 @@
         <f>M8-I9</f>
         <v>484757.02999999991</v>
       </c>
-      <c r="O9" s="104" t="s">
+      <c r="O9" s="98" t="s">
         <v>87</v>
       </c>
-      <c r="P9" s="104"/>
-      <c r="Q9" s="104"/>
+      <c r="P9" s="98"/>
+      <c r="Q9" s="98"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="81" t="s">
@@ -5782,11 +6413,11 @@
         <f t="shared" ref="M10:M63" si="2">M9-I10</f>
         <v>475943.2699999999</v>
       </c>
-      <c r="O10" s="105" t="s">
+      <c r="O10" s="99" t="s">
         <v>88</v>
       </c>
-      <c r="P10" s="105"/>
-      <c r="Q10" s="105"/>
+      <c r="P10" s="99"/>
+      <c r="Q10" s="99"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="81" t="s">
@@ -5828,11 +6459,11 @@
         <f t="shared" si="2"/>
         <v>467129.50999999989</v>
       </c>
-      <c r="O11" s="106" t="s">
+      <c r="O11" s="100" t="s">
         <v>90</v>
       </c>
-      <c r="P11" s="106"/>
-      <c r="Q11" s="106"/>
+      <c r="P11" s="100"/>
+      <c r="Q11" s="100"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="83" t="s">
@@ -7430,7 +8061,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B1:R125"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -7638,10 +8269,10 @@
         <f>M5-I6</f>
         <v>1073254.2800000003</v>
       </c>
-      <c r="O6" s="103" t="s">
+      <c r="O6" s="97" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="103"/>
+      <c r="P6" s="97"/>
       <c r="Q6" s="82">
         <f>Q4/O4-1</f>
         <v>-0.3333332612783364</v>
@@ -7816,11 +8447,11 @@
         <f t="shared" si="2"/>
         <v>999236.76000000036</v>
       </c>
-      <c r="O10" s="104" t="s">
+      <c r="O10" s="98" t="s">
         <v>87</v>
       </c>
-      <c r="P10" s="104"/>
-      <c r="Q10" s="104"/>
+      <c r="P10" s="98"/>
+      <c r="Q10" s="98"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="79" t="s">
@@ -7862,11 +8493,11 @@
         <f t="shared" si="2"/>
         <v>980732.38000000035</v>
       </c>
-      <c r="O11" s="105" t="s">
+      <c r="O11" s="99" t="s">
         <v>88</v>
       </c>
-      <c r="P11" s="105"/>
-      <c r="Q11" s="105"/>
+      <c r="P11" s="99"/>
+      <c r="Q11" s="99"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="79" t="s">
@@ -10538,7 +11169,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{076A243B-6594-4F6F-90C2-83485C35A53B}">
   <dimension ref="B1:R85"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -10748,10 +11379,10 @@
         <f>M5-I6</f>
         <v>1727211.77</v>
       </c>
-      <c r="O6" s="103" t="s">
+      <c r="O6" s="97" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="103"/>
+      <c r="P6" s="97"/>
       <c r="Q6" s="82">
         <f>(Q4/O4)-1</f>
         <v>-0.23333330852134659</v>
@@ -10882,11 +11513,11 @@
         <f t="shared" ref="M9:M63" si="2">M8-I9</f>
         <v>1637873.24</v>
       </c>
-      <c r="O9" s="104" t="s">
+      <c r="O9" s="98" t="s">
         <v>87</v>
       </c>
-      <c r="P9" s="104"/>
-      <c r="Q9" s="104"/>
+      <c r="P9" s="98"/>
+      <c r="Q9" s="98"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="81" t="s">
@@ -10928,11 +11559,11 @@
         <f t="shared" si="2"/>
         <v>1608093.73</v>
       </c>
-      <c r="O10" s="105" t="s">
+      <c r="O10" s="99" t="s">
         <v>88</v>
       </c>
-      <c r="P10" s="105"/>
-      <c r="Q10" s="105"/>
+      <c r="P10" s="99"/>
+      <c r="Q10" s="99"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="81" t="s">
@@ -10974,11 +11605,11 @@
         <f t="shared" si="2"/>
         <v>1578314.22</v>
       </c>
-      <c r="O11" s="106" t="s">
+      <c r="O11" s="100" t="s">
         <v>90</v>
       </c>
-      <c r="P11" s="106"/>
-      <c r="Q11" s="106"/>
+      <c r="P11" s="100"/>
+      <c r="Q11" s="100"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="81" t="s">
@@ -12568,7 +13199,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08920BEF-61AE-469B-8613-B03EE9E56473}">
   <dimension ref="B1:R85"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -12750,10 +13381,10 @@
         <f>M5-I6</f>
         <v>88254.450000000012</v>
       </c>
-      <c r="O6" s="103" t="s">
+      <c r="O6" s="97" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="103"/>
+      <c r="P6" s="97"/>
       <c r="Q6" s="82">
         <f>(Q4/O4)-1</f>
         <v>-0.14999919494129588</v>
@@ -12839,11 +13470,11 @@
         <f t="shared" ref="M9:M63" si="2">M8-I9</f>
         <v>83689.590000000026</v>
       </c>
-      <c r="O9" s="104" t="s">
+      <c r="O9" s="98" t="s">
         <v>87</v>
       </c>
-      <c r="P9" s="104"/>
-      <c r="Q9" s="104"/>
+      <c r="P9" s="98"/>
+      <c r="Q9" s="98"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="39"/>
@@ -12870,11 +13501,11 @@
         <f t="shared" si="2"/>
         <v>82167.97000000003</v>
       </c>
-      <c r="O10" s="105" t="s">
+      <c r="O10" s="99" t="s">
         <v>88</v>
       </c>
-      <c r="P10" s="105"/>
-      <c r="Q10" s="105"/>
+      <c r="P10" s="99"/>
+      <c r="Q10" s="99"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="39"/>
@@ -12901,11 +13532,11 @@
         <f t="shared" si="2"/>
         <v>80646.350000000035</v>
       </c>
-      <c r="O11" s="106" t="s">
+      <c r="O11" s="100" t="s">
         <v>90</v>
       </c>
-      <c r="P11" s="106"/>
-      <c r="Q11" s="106"/>
+      <c r="P11" s="100"/>
+      <c r="Q11" s="100"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="39"/>
@@ -14399,7 +15030,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00D981B1-E026-41C2-8293-91583FAD4939}">
   <dimension ref="B1:R58"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -14567,10 +15198,10 @@
         <f>M5-I6</f>
         <v>-501.4</v>
       </c>
-      <c r="O6" s="103" t="s">
+      <c r="O6" s="97" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="103"/>
+      <c r="P6" s="97"/>
       <c r="Q6" s="82">
         <f>(Q4/O4)-1</f>
         <v>-0.33618406919008692</v>
@@ -15581,7 +16212,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D05F36B-D5CF-4328-B814-E173D67EEF77}">
   <dimension ref="B1:Z28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -16525,7 +17156,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{420301BD-1EC9-404C-9D58-1869DDAA2327}">
   <dimension ref="B2:P9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
data(sar): atualizacao automatica da base SAR via rede local
</commit_message>
<xml_diff>
--- a/parcelamentos_local.xlsx
+++ b/parcelamentos_local.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\10.121.21.252\controladoria\Vitor\TRIBUTARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{469E9222-E42F-478F-B55E-489D032C95AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3F9CF56-881C-45B9-A69C-14C3D94E8347}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="804" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="804" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SALDO CREDOR INSS" sheetId="14" r:id="rId1"/>
@@ -105,7 +105,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="114">
   <si>
     <t>TAURA AGRONEGOCIOS - IMPOSTOS EM ABERTO - NÃO PARCELADOS NA RECEITA FEDERAL</t>
   </si>
@@ -447,9 +447,6 @@
   </si>
   <si>
     <t>Status</t>
-  </si>
-  <si>
-    <t>Pendente</t>
   </si>
 </sst>
 </file>
@@ -1012,7 +1009,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="140">
+  <cellXfs count="139">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1263,7 +1260,7 @@
     <xf numFmtId="43" fontId="21" fillId="8" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1282,9 +1279,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -5023,10 +5017,10 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="97"/>
-      <c r="B8" s="129" t="s">
+      <c r="B8" s="122" t="s">
         <v>101</v>
       </c>
-      <c r="C8" s="129"/>
+      <c r="C8" s="122"/>
       <c r="D8" s="103"/>
       <c r="E8" s="103"/>
       <c r="F8" s="103"/>
@@ -5743,7 +5737,7 @@
       </c>
       <c r="C15" s="17">
         <f>'PARCELAMENTO SC'!R4</f>
-        <v>3855.700000000008</v>
+        <v>0</v>
       </c>
       <c r="D15" s="18" t="s">
         <v>111</v>
@@ -5759,7 +5753,7 @@
       <c r="B16" s="20"/>
       <c r="C16" s="89">
         <f>SUM(C11:C15)</f>
-        <v>2376964.6699999995</v>
+        <v>2373108.9699999993</v>
       </c>
       <c r="D16" s="20"/>
       <c r="E16" s="20"/>
@@ -6300,10 +6294,10 @@
         <f>M5-I6</f>
         <v>511198.30999999994</v>
       </c>
-      <c r="O6" s="130" t="s">
+      <c r="O6" s="129" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="130"/>
+      <c r="P6" s="129"/>
       <c r="Q6" s="82">
         <f>(Q4/O4)-1</f>
         <v>-0.46666646370129106</v>
@@ -6434,11 +6428,11 @@
         <f>M8-I9</f>
         <v>484757.02999999991</v>
       </c>
-      <c r="O9" s="131" t="s">
+      <c r="O9" s="130" t="s">
         <v>87</v>
       </c>
-      <c r="P9" s="131"/>
-      <c r="Q9" s="131"/>
+      <c r="P9" s="130"/>
+      <c r="Q9" s="130"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="81" t="s">
@@ -6480,11 +6474,11 @@
         <f t="shared" ref="M10:M63" si="2">M9-I10</f>
         <v>475943.2699999999</v>
       </c>
-      <c r="O10" s="132" t="s">
+      <c r="O10" s="131" t="s">
         <v>88</v>
       </c>
-      <c r="P10" s="132"/>
-      <c r="Q10" s="132"/>
+      <c r="P10" s="131"/>
+      <c r="Q10" s="131"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="81" t="s">
@@ -6526,11 +6520,11 @@
         <f t="shared" si="2"/>
         <v>467129.50999999989</v>
       </c>
-      <c r="O11" s="133" t="s">
+      <c r="O11" s="132" t="s">
         <v>90</v>
       </c>
-      <c r="P11" s="133"/>
-      <c r="Q11" s="133"/>
+      <c r="P11" s="132"/>
+      <c r="Q11" s="132"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="83" t="s">
@@ -8340,10 +8334,10 @@
         <f>M5-I6</f>
         <v>1073254.2800000003</v>
       </c>
-      <c r="O6" s="130" t="s">
+      <c r="O6" s="129" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="130"/>
+      <c r="P6" s="129"/>
       <c r="Q6" s="82">
         <f>Q4/O4-1</f>
         <v>-0.36666658740617009</v>
@@ -8472,11 +8466,11 @@
         <f t="shared" si="2"/>
         <v>1017741.1400000004</v>
       </c>
-      <c r="O9" s="134" t="s">
+      <c r="O9" s="133" t="s">
         <v>86</v>
       </c>
-      <c r="P9" s="134"/>
-      <c r="Q9" s="134"/>
+      <c r="P9" s="133"/>
+      <c r="Q9" s="133"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="79" t="s">
@@ -8518,11 +8512,11 @@
         <f t="shared" si="2"/>
         <v>999236.76000000036</v>
       </c>
-      <c r="O10" s="131" t="s">
+      <c r="O10" s="130" t="s">
         <v>87</v>
       </c>
-      <c r="P10" s="131"/>
-      <c r="Q10" s="131"/>
+      <c r="P10" s="130"/>
+      <c r="Q10" s="130"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="79" t="s">
@@ -8564,11 +8558,11 @@
         <f t="shared" si="2"/>
         <v>980732.38000000035</v>
       </c>
-      <c r="O11" s="132" t="s">
+      <c r="O11" s="131" t="s">
         <v>88</v>
       </c>
-      <c r="P11" s="132"/>
-      <c r="Q11" s="132"/>
+      <c r="P11" s="131"/>
+      <c r="Q11" s="131"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="79" t="s">
@@ -11460,10 +11454,10 @@
         <f>M5-I6</f>
         <v>1727211.77</v>
       </c>
-      <c r="O6" s="130" t="s">
+      <c r="O6" s="129" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="130"/>
+      <c r="P6" s="129"/>
       <c r="Q6" s="82">
         <f>(Q4/O4)-1</f>
         <v>-0.26666663831011039</v>
@@ -11594,11 +11588,11 @@
         <f t="shared" ref="M9:M63" si="2">M8-I9</f>
         <v>1637873.24</v>
       </c>
-      <c r="O9" s="131" t="s">
+      <c r="O9" s="130" t="s">
         <v>87</v>
       </c>
-      <c r="P9" s="131"/>
-      <c r="Q9" s="131"/>
+      <c r="P9" s="130"/>
+      <c r="Q9" s="130"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="81" t="s">
@@ -11640,11 +11634,11 @@
         <f t="shared" si="2"/>
         <v>1608093.73</v>
       </c>
-      <c r="O10" s="132" t="s">
+      <c r="O10" s="131" t="s">
         <v>88</v>
       </c>
-      <c r="P10" s="132"/>
-      <c r="Q10" s="132"/>
+      <c r="P10" s="131"/>
+      <c r="Q10" s="131"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="81" t="s">
@@ -11686,11 +11680,11 @@
         <f t="shared" si="2"/>
         <v>1578314.22</v>
       </c>
-      <c r="O11" s="133" t="s">
+      <c r="O11" s="132" t="s">
         <v>90</v>
       </c>
-      <c r="P11" s="133"/>
-      <c r="Q11" s="133"/>
+      <c r="P11" s="132"/>
+      <c r="Q11" s="132"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="81" t="s">
@@ -13466,10 +13460,10 @@
         <f>M5-I6</f>
         <v>88254.450000000012</v>
       </c>
-      <c r="O6" s="130" t="s">
+      <c r="O6" s="129" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="130"/>
+      <c r="P6" s="129"/>
       <c r="Q6" s="82">
         <f>(Q4/O4)-1</f>
         <v>-0.14999919494129588</v>
@@ -13555,11 +13549,11 @@
         <f t="shared" ref="M9:M63" si="2">M8-I9</f>
         <v>83689.590000000026</v>
       </c>
-      <c r="O9" s="131" t="s">
+      <c r="O9" s="130" t="s">
         <v>87</v>
       </c>
-      <c r="P9" s="131"/>
-      <c r="Q9" s="131"/>
+      <c r="P9" s="130"/>
+      <c r="Q9" s="130"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="39"/>
@@ -13586,11 +13580,11 @@
         <f t="shared" si="2"/>
         <v>82167.97000000003</v>
       </c>
-      <c r="O10" s="132" t="s">
+      <c r="O10" s="131" t="s">
         <v>88</v>
       </c>
-      <c r="P10" s="132"/>
-      <c r="Q10" s="132"/>
+      <c r="P10" s="131"/>
+      <c r="Q10" s="131"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="39"/>
@@ -13617,11 +13611,11 @@
         <f t="shared" si="2"/>
         <v>80646.350000000035</v>
       </c>
-      <c r="O11" s="133" t="s">
+      <c r="O11" s="132" t="s">
         <v>90</v>
       </c>
-      <c r="P11" s="133"/>
-      <c r="Q11" s="133"/>
+      <c r="P11" s="132"/>
+      <c r="Q11" s="132"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="39"/>
@@ -15232,15 +15226,15 @@
       </c>
       <c r="P4" s="32">
         <f>I52</f>
-        <v>10105.300000000005</v>
+        <v>11562</v>
       </c>
       <c r="Q4" s="33">
-        <f>K5+K6+K7+K8+K9+K10+K11+K12+K13+K14+K15+K16+K17+K18+K19+K20+K21+K22+K23+K24+K25+K26+K27+K28+K29+K30+K31+K32</f>
-        <v>6249.5999999999967</v>
+        <f>K5+K6+K7+K8+K9+K10+K11+K12+K13+K14+K15+K16+K17+K18+K19+K20+K21+K22+K23+K24+K25+K26+K27+K28+K29+K30+K31+K32+K33+K34+K35+K36+K37+K38+K39+K40+K41+K42+K43+K44+K45+K46+K47+K48+K49+K50+K51</f>
+        <v>11562.000000000004</v>
       </c>
       <c r="R4" s="34">
         <f>P4-Q4</f>
-        <v>3855.700000000008</v>
+        <v>0</v>
       </c>
       <c r="S4" s="34">
         <f>J5+J6+J7+J8+J9+J10+J11+J12+J13+J14+J15+J16+J17+J18+J19+J20+J21+J22+J23+J24+J25+J26+J27+J28+J29+J30+J31+J32+J33+J34+J35+J36+J37+J38+J39+J40+J41+J42+J43+J44+J45+J46+J47+J48+J49+J50+J51-354.74</f>
@@ -15270,7 +15264,7 @@
       </c>
       <c r="M5" s="31">
         <f>$P$4-I4</f>
-        <v>9894.7700000000041</v>
+        <v>11351.47</v>
       </c>
       <c r="N5" s="84" t="s">
         <v>25</v>
@@ -15299,18 +15293,18 @@
       </c>
       <c r="M6" s="31">
         <f>M5-I6</f>
-        <v>9684.2400000000034</v>
+        <v>11140.939999999999</v>
       </c>
       <c r="N6" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="P6" s="130" t="s">
+      <c r="P6" s="129" t="s">
         <v>89</v>
       </c>
-      <c r="Q6" s="130"/>
+      <c r="Q6" s="129"/>
       <c r="R6" s="82">
         <f>(R4/P4)-1</f>
-        <v>-0.61844774524259494</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="7" spans="2:19" customFormat="1" x14ac:dyDescent="0.3">
@@ -15336,7 +15330,7 @@
       </c>
       <c r="M7" s="31">
         <f t="shared" ref="M7:M51" si="1">M6-I7</f>
-        <v>9473.7100000000028</v>
+        <v>10930.409999999998</v>
       </c>
       <c r="N7" s="84" t="s">
         <v>25</v>
@@ -15368,10 +15362,14 @@
       </c>
       <c r="M8" s="31">
         <f t="shared" si="1"/>
-        <v>9263.1800000000021</v>
+        <v>10719.879999999997</v>
       </c>
       <c r="N8" s="84" t="s">
         <v>25</v>
+      </c>
+      <c r="R8" s="88">
+        <f>Q4-P4</f>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="2:19" customFormat="1" x14ac:dyDescent="0.3">
@@ -15397,14 +15395,14 @@
       </c>
       <c r="M9" s="31">
         <f t="shared" si="1"/>
-        <v>9052.6500000000015</v>
+        <v>10509.349999999997</v>
       </c>
       <c r="N9" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="P9" s="135"/>
-      <c r="Q9" s="135"/>
-      <c r="R9" s="135"/>
+      <c r="P9" s="134"/>
+      <c r="Q9" s="134"/>
+      <c r="R9" s="134"/>
     </row>
     <row r="10" spans="2:19" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="39"/>
@@ -15429,14 +15427,14 @@
       </c>
       <c r="M10" s="31">
         <f t="shared" si="1"/>
-        <v>8842.1200000000008</v>
+        <v>10298.819999999996</v>
       </c>
       <c r="N10" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="P10" s="135"/>
-      <c r="Q10" s="135"/>
-      <c r="R10" s="135"/>
+      <c r="P10" s="134"/>
+      <c r="Q10" s="134"/>
+      <c r="R10" s="134"/>
     </row>
     <row r="11" spans="2:19" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="39"/>
@@ -15461,14 +15459,14 @@
       </c>
       <c r="M11" s="31">
         <f t="shared" si="1"/>
-        <v>8631.59</v>
+        <v>10088.289999999995</v>
       </c>
       <c r="N11" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="P11" s="135"/>
-      <c r="Q11" s="135"/>
-      <c r="R11" s="135"/>
+      <c r="P11" s="134"/>
+      <c r="Q11" s="134"/>
+      <c r="R11" s="134"/>
     </row>
     <row r="12" spans="2:19" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="39"/>
@@ -15493,7 +15491,7 @@
       </c>
       <c r="M12" s="31">
         <f t="shared" si="1"/>
-        <v>8421.06</v>
+        <v>9877.7599999999948</v>
       </c>
       <c r="N12" s="84" t="s">
         <v>25</v>
@@ -15522,7 +15520,7 @@
       </c>
       <c r="M13" s="31">
         <f t="shared" si="1"/>
-        <v>8210.5299999999988</v>
+        <v>9667.2299999999941</v>
       </c>
       <c r="N13" s="84" t="s">
         <v>25</v>
@@ -15551,7 +15549,7 @@
       </c>
       <c r="M14" s="31">
         <f t="shared" si="1"/>
-        <v>7999.9999999999991</v>
+        <v>9456.6999999999935</v>
       </c>
       <c r="N14" s="84" t="s">
         <v>25</v>
@@ -15580,7 +15578,7 @@
       </c>
       <c r="M15" s="31">
         <f t="shared" si="1"/>
-        <v>7789.4699999999993</v>
+        <v>9246.1699999999928</v>
       </c>
       <c r="N15" s="84" t="s">
         <v>25</v>
@@ -15608,7 +15606,7 @@
       </c>
       <c r="M16" s="31">
         <f t="shared" si="1"/>
-        <v>7578.94</v>
+        <v>9035.6399999999921</v>
       </c>
       <c r="N16" s="84" t="s">
         <v>25</v>
@@ -15636,7 +15634,7 @@
       </c>
       <c r="M17" s="31">
         <f t="shared" si="1"/>
-        <v>7368.41</v>
+        <v>8825.1099999999915</v>
       </c>
       <c r="N17" s="84" t="s">
         <v>25</v>
@@ -15664,7 +15662,7 @@
       </c>
       <c r="M18" s="31">
         <f t="shared" si="1"/>
-        <v>7157.88</v>
+        <v>8614.5799999999908</v>
       </c>
       <c r="N18" s="84" t="s">
         <v>25</v>
@@ -15692,7 +15690,7 @@
       </c>
       <c r="M19" s="31">
         <f t="shared" si="1"/>
-        <v>6947.35</v>
+        <v>8404.0499999999902</v>
       </c>
       <c r="N19" s="84" t="s">
         <v>25</v>
@@ -15720,7 +15718,7 @@
       </c>
       <c r="M20" s="31">
         <f t="shared" si="1"/>
-        <v>6736.8200000000006</v>
+        <v>8193.5199999999895</v>
       </c>
       <c r="N20" s="84" t="s">
         <v>25</v>
@@ -15748,7 +15746,7 @@
       </c>
       <c r="M21" s="31">
         <f t="shared" si="1"/>
-        <v>6526.2900000000009</v>
+        <v>7982.9899999999898</v>
       </c>
       <c r="N21" s="84" t="s">
         <v>25</v>
@@ -15776,7 +15774,7 @@
       </c>
       <c r="M22" s="31">
         <f t="shared" si="1"/>
-        <v>6315.7600000000011</v>
+        <v>7772.45999999999</v>
       </c>
       <c r="N22" s="84" t="s">
         <v>25</v>
@@ -15804,7 +15802,7 @@
       </c>
       <c r="M23" s="31">
         <f t="shared" si="1"/>
-        <v>6105.2300000000014</v>
+        <v>7561.9299999999903</v>
       </c>
       <c r="N23" s="84" t="s">
         <v>25</v>
@@ -15832,7 +15830,7 @@
       </c>
       <c r="M24" s="31">
         <f t="shared" si="1"/>
-        <v>5894.7000000000016</v>
+        <v>7351.3999999999905</v>
       </c>
       <c r="N24" s="84" t="s">
         <v>25</v>
@@ -15860,7 +15858,7 @@
       </c>
       <c r="M25" s="31">
         <f t="shared" si="1"/>
-        <v>5684.1700000000019</v>
+        <v>7140.8699999999908</v>
       </c>
       <c r="N25" s="84" t="s">
         <v>25</v>
@@ -15888,7 +15886,7 @@
       </c>
       <c r="M26" s="31">
         <f t="shared" si="1"/>
-        <v>5473.6400000000021</v>
+        <v>6930.3399999999911</v>
       </c>
       <c r="N26" s="84" t="s">
         <v>25</v>
@@ -15916,7 +15914,7 @@
       </c>
       <c r="M27" s="31">
         <f t="shared" si="1"/>
-        <v>5263.1100000000024</v>
+        <v>6719.8099999999913</v>
       </c>
       <c r="N27" s="84" t="s">
         <v>25</v>
@@ -15944,7 +15942,7 @@
       </c>
       <c r="M28" s="31">
         <f t="shared" si="1"/>
-        <v>5052.5800000000027</v>
+        <v>6509.2799999999916</v>
       </c>
       <c r="N28" s="84" t="s">
         <v>25</v>
@@ -15972,7 +15970,7 @@
       </c>
       <c r="M29" s="31">
         <f t="shared" si="1"/>
-        <v>4842.0500000000029</v>
+        <v>6298.7499999999918</v>
       </c>
       <c r="N29" s="84" t="s">
         <v>25</v>
@@ -16000,7 +15998,7 @@
       </c>
       <c r="M30" s="31">
         <f t="shared" si="1"/>
-        <v>4631.5200000000032</v>
+        <v>6088.2199999999921</v>
       </c>
       <c r="N30" s="84" t="s">
         <v>25</v>
@@ -16028,7 +16026,7 @@
       </c>
       <c r="M31" s="31">
         <f t="shared" si="1"/>
-        <v>4420.9900000000034</v>
+        <v>5877.6899999999923</v>
       </c>
       <c r="N31" s="84" t="s">
         <v>25</v>
@@ -16056,7 +16054,7 @@
       </c>
       <c r="M32" s="31">
         <f t="shared" si="1"/>
-        <v>4210.4600000000037</v>
+        <v>5667.1599999999926</v>
       </c>
       <c r="N32" s="84" t="s">
         <v>25</v>
@@ -16084,10 +16082,10 @@
       </c>
       <c r="M33" s="31">
         <f t="shared" si="1"/>
-        <v>3999.9300000000035</v>
-      </c>
-      <c r="N33" s="122" t="s">
-        <v>114</v>
+        <v>5456.6299999999928</v>
+      </c>
+      <c r="N33" s="84" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="34" spans="3:14" x14ac:dyDescent="0.3">
@@ -16112,10 +16110,10 @@
       </c>
       <c r="M34" s="31">
         <f t="shared" si="1"/>
-        <v>3789.4000000000033</v>
-      </c>
-      <c r="N34" s="122" t="s">
-        <v>114</v>
+        <v>5246.0999999999931</v>
+      </c>
+      <c r="N34" s="84" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="35" spans="3:14" x14ac:dyDescent="0.3">
@@ -16140,10 +16138,10 @@
       </c>
       <c r="M35" s="31">
         <f t="shared" si="1"/>
-        <v>3578.8700000000031</v>
-      </c>
-      <c r="N35" s="122" t="s">
-        <v>114</v>
+        <v>5035.5699999999933</v>
+      </c>
+      <c r="N35" s="84" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="36" spans="3:14" x14ac:dyDescent="0.3">
@@ -16168,10 +16166,10 @@
       </c>
       <c r="M36" s="31">
         <f t="shared" si="1"/>
-        <v>3368.3400000000029</v>
-      </c>
-      <c r="N36" s="122" t="s">
-        <v>114</v>
+        <v>4825.0399999999936</v>
+      </c>
+      <c r="N36" s="84" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="37" spans="3:14" x14ac:dyDescent="0.3">
@@ -16196,10 +16194,10 @@
       </c>
       <c r="M37" s="31">
         <f t="shared" si="1"/>
-        <v>3157.8100000000027</v>
-      </c>
-      <c r="N37" s="122" t="s">
-        <v>114</v>
+        <v>4614.5099999999939</v>
+      </c>
+      <c r="N37" s="84" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="38" spans="3:14" x14ac:dyDescent="0.3">
@@ -16224,10 +16222,10 @@
       </c>
       <c r="M38" s="31">
         <f t="shared" si="1"/>
-        <v>2947.2800000000025</v>
-      </c>
-      <c r="N38" s="122" t="s">
-        <v>114</v>
+        <v>4403.9799999999941</v>
+      </c>
+      <c r="N38" s="84" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="39" spans="3:14" x14ac:dyDescent="0.3">
@@ -16252,10 +16250,10 @@
       </c>
       <c r="M39" s="31">
         <f t="shared" si="1"/>
-        <v>2736.7500000000023</v>
-      </c>
-      <c r="N39" s="122" t="s">
-        <v>114</v>
+        <v>4193.4499999999944</v>
+      </c>
+      <c r="N39" s="84" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="40" spans="3:14" x14ac:dyDescent="0.3">
@@ -16280,10 +16278,10 @@
       </c>
       <c r="M40" s="31">
         <f t="shared" si="1"/>
-        <v>2526.2200000000021</v>
-      </c>
-      <c r="N40" s="122" t="s">
-        <v>114</v>
+        <v>3982.9199999999942</v>
+      </c>
+      <c r="N40" s="84" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="41" spans="3:14" x14ac:dyDescent="0.3">
@@ -16308,10 +16306,10 @@
       </c>
       <c r="M41" s="31">
         <f t="shared" si="1"/>
-        <v>2315.6900000000019</v>
-      </c>
-      <c r="N41" s="122" t="s">
-        <v>114</v>
+        <v>3772.389999999994</v>
+      </c>
+      <c r="N41" s="84" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="42" spans="3:14" x14ac:dyDescent="0.3">
@@ -16336,10 +16334,10 @@
       </c>
       <c r="M42" s="31">
         <f t="shared" si="1"/>
-        <v>2105.1600000000017</v>
-      </c>
-      <c r="N42" s="122" t="s">
-        <v>114</v>
+        <v>3561.8599999999938</v>
+      </c>
+      <c r="N42" s="84" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="43" spans="3:14" x14ac:dyDescent="0.3">
@@ -16364,10 +16362,10 @@
       </c>
       <c r="M43" s="31">
         <f t="shared" si="1"/>
-        <v>1894.6300000000017</v>
-      </c>
-      <c r="N43" s="122" t="s">
-        <v>114</v>
+        <v>3351.3299999999936</v>
+      </c>
+      <c r="N43" s="84" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="44" spans="3:14" x14ac:dyDescent="0.3">
@@ -16392,10 +16390,10 @@
       </c>
       <c r="M44" s="31">
         <f t="shared" si="1"/>
-        <v>1684.1000000000017</v>
-      </c>
-      <c r="N44" s="122" t="s">
-        <v>114</v>
+        <v>3140.7999999999934</v>
+      </c>
+      <c r="N44" s="84" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="45" spans="3:14" x14ac:dyDescent="0.3">
@@ -16420,10 +16418,10 @@
       </c>
       <c r="M45" s="31">
         <f t="shared" si="1"/>
-        <v>1473.5700000000018</v>
-      </c>
-      <c r="N45" s="122" t="s">
-        <v>114</v>
+        <v>2930.2699999999932</v>
+      </c>
+      <c r="N45" s="84" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="46" spans="3:14" x14ac:dyDescent="0.3">
@@ -16448,10 +16446,10 @@
       </c>
       <c r="M46" s="31">
         <f t="shared" si="1"/>
-        <v>1263.0400000000018</v>
-      </c>
-      <c r="N46" s="122" t="s">
-        <v>114</v>
+        <v>2719.739999999993</v>
+      </c>
+      <c r="N46" s="84" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="47" spans="3:14" x14ac:dyDescent="0.3">
@@ -16476,10 +16474,10 @@
       </c>
       <c r="M47" s="31">
         <f t="shared" si="1"/>
-        <v>1052.5100000000018</v>
-      </c>
-      <c r="N47" s="122" t="s">
-        <v>114</v>
+        <v>2509.2099999999928</v>
+      </c>
+      <c r="N47" s="84" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="48" spans="3:14" x14ac:dyDescent="0.3">
@@ -16504,10 +16502,10 @@
       </c>
       <c r="M48" s="31">
         <f t="shared" si="1"/>
-        <v>841.98000000000184</v>
-      </c>
-      <c r="N48" s="122" t="s">
-        <v>114</v>
+        <v>2298.6799999999926</v>
+      </c>
+      <c r="N48" s="84" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="49" spans="3:14" x14ac:dyDescent="0.3">
@@ -16532,10 +16530,10 @@
       </c>
       <c r="M49" s="31">
         <f t="shared" si="1"/>
-        <v>631.45000000000186</v>
-      </c>
-      <c r="N49" s="122" t="s">
-        <v>114</v>
+        <v>2088.1499999999924</v>
+      </c>
+      <c r="N49" s="84" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="50" spans="3:14" x14ac:dyDescent="0.3">
@@ -16560,10 +16558,10 @@
       </c>
       <c r="M50" s="31">
         <f t="shared" si="1"/>
-        <v>420.92000000000189</v>
-      </c>
-      <c r="N50" s="122" t="s">
-        <v>114</v>
+        <v>1877.6199999999924</v>
+      </c>
+      <c r="N50" s="84" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="51" spans="3:14" x14ac:dyDescent="0.3">
@@ -16588,10 +16586,10 @@
       </c>
       <c r="M51" s="31">
         <f t="shared" si="1"/>
-        <v>210.39000000000189</v>
-      </c>
-      <c r="N51" s="122" t="s">
-        <v>114</v>
+        <v>1667.0899999999924</v>
+      </c>
+      <c r="N51" s="84" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="52" spans="3:14" x14ac:dyDescent="0.3">
@@ -16602,8 +16600,8 @@
       <c r="G52" s="42"/>
       <c r="H52" s="42"/>
       <c r="I52" s="42">
-        <f>SUM(I4:I51)-0.14</f>
-        <v>10105.300000000005</v>
+        <f>SUM(I4:I51)-0.14+J33+J34+J35+J36+J37+J38+J39+J40+J41+J42+J43+J44+J45+J46+J47+J48+J49+J50+J51+144.37</f>
+        <v>11562</v>
       </c>
       <c r="J52" s="42"/>
       <c r="K52" s="42"/>
@@ -16715,30 +16713,30 @@
   <sheetData>
     <row r="1" spans="2:26" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:26" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="137" t="s">
+      <c r="B2" s="136" t="s">
         <v>52</v>
       </c>
-      <c r="C2" s="138"/>
-      <c r="D2" s="138"/>
-      <c r="E2" s="138"/>
-      <c r="F2" s="138"/>
-      <c r="G2" s="138"/>
-      <c r="H2" s="138"/>
-      <c r="I2" s="138"/>
-      <c r="J2" s="138"/>
-      <c r="K2" s="138"/>
-      <c r="L2" s="138"/>
-      <c r="M2" s="138"/>
-      <c r="N2" s="138"/>
-      <c r="O2" s="138"/>
-      <c r="P2" s="138"/>
-      <c r="Q2" s="138"/>
-      <c r="R2" s="138"/>
-      <c r="S2" s="138"/>
-      <c r="T2" s="138"/>
-      <c r="U2" s="138"/>
-      <c r="V2" s="138"/>
-      <c r="W2" s="139"/>
+      <c r="C2" s="137"/>
+      <c r="D2" s="137"/>
+      <c r="E2" s="137"/>
+      <c r="F2" s="137"/>
+      <c r="G2" s="137"/>
+      <c r="H2" s="137"/>
+      <c r="I2" s="137"/>
+      <c r="J2" s="137"/>
+      <c r="K2" s="137"/>
+      <c r="L2" s="137"/>
+      <c r="M2" s="137"/>
+      <c r="N2" s="137"/>
+      <c r="O2" s="137"/>
+      <c r="P2" s="137"/>
+      <c r="Q2" s="137"/>
+      <c r="R2" s="137"/>
+      <c r="S2" s="137"/>
+      <c r="T2" s="137"/>
+      <c r="U2" s="137"/>
+      <c r="V2" s="137"/>
+      <c r="W2" s="138"/>
     </row>
     <row r="3" spans="2:26" s="4" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="48" t="s">
@@ -17569,8 +17567,8 @@
       <c r="Z22" s="57"/>
     </row>
     <row r="24" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="P24" s="136"/>
-      <c r="Q24" s="136"/>
+      <c r="P24" s="135"/>
+      <c r="Q24" s="135"/>
       <c r="R24" s="73"/>
       <c r="S24" s="73"/>
       <c r="T24" s="73"/>
@@ -17579,8 +17577,8 @@
       <c r="W24" s="74"/>
     </row>
     <row r="25" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="P25" s="136"/>
-      <c r="Q25" s="136"/>
+      <c r="P25" s="135"/>
+      <c r="Q25" s="135"/>
       <c r="R25" s="73"/>
       <c r="S25" s="73"/>
       <c r="T25" s="73"/>
@@ -17589,8 +17587,8 @@
       <c r="W25" s="74"/>
     </row>
     <row r="26" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="P26" s="136"/>
-      <c r="Q26" s="136"/>
+      <c r="P26" s="135"/>
+      <c r="Q26" s="135"/>
       <c r="R26" s="73"/>
       <c r="S26" s="73"/>
       <c r="T26" s="73"/>
@@ -17599,8 +17597,8 @@
       <c r="W26" s="74"/>
     </row>
     <row r="27" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="P27" s="136"/>
-      <c r="Q27" s="136"/>
+      <c r="P27" s="135"/>
+      <c r="Q27" s="135"/>
       <c r="R27" s="73"/>
       <c r="S27" s="73"/>
       <c r="T27" s="73"/>
@@ -17609,8 +17607,8 @@
       <c r="W27" s="75"/>
     </row>
     <row r="28" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="P28" s="136"/>
-      <c r="Q28" s="136"/>
+      <c r="P28" s="135"/>
+      <c r="Q28" s="135"/>
       <c r="R28" s="73"/>
       <c r="S28" s="73"/>
       <c r="T28" s="73"/>

</xml_diff>

<commit_message>
data(impostos): atualizacao automatica da base tributaria e parcelamentos
</commit_message>
<xml_diff>
--- a/parcelamentos_local.xlsx
+++ b/parcelamentos_local.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\10.121.21.252\controladoria\Vitor\TRIBUTARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3F9CF56-881C-45B9-A69C-14C3D94E8347}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A96A1E39-68A3-4984-8191-C9CAFE0E0404}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="804" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="804" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SALDO CREDOR INSS" sheetId="14" r:id="rId1"/>
@@ -1260,6 +1260,12 @@
     <xf numFmtId="43" fontId="21" fillId="8" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1281,9 +1287,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1294,9 +1297,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2798,10 +2798,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$Q$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$R$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="15"/>
+                <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -2846,16 +2846,19 @@
                 </c:pt>
                 <c:pt idx="14">
                   <c:v>46266</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>46296</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$3:$Q$3</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$3:$R$3</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="15"/>
+                <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>4720740.33</c:v>
                 </c:pt>
@@ -2900,6 +2903,9 @@
                 </c:pt>
                 <c:pt idx="14">
                   <c:v>3796974.4</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>3713217.08</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2936,10 +2942,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$Q$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$R$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="15"/>
+                <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -2984,6 +2990,9 @@
                 </c:pt>
                 <c:pt idx="14">
                   <c:v>46266</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>46296</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3071,10 +3080,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$Q$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$R$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="15"/>
+                <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -3119,6 +3128,9 @@
                 </c:pt>
                 <c:pt idx="14">
                   <c:v>46266</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>46296</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3206,10 +3218,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$Q$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$R$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="15"/>
+                <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -3254,6 +3266,9 @@
                 </c:pt>
                 <c:pt idx="14">
                   <c:v>46266</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>46296</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3344,10 +3359,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$Q$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$R$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="15"/>
+                <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -3392,6 +3407,9 @@
                 </c:pt>
                 <c:pt idx="14">
                   <c:v>46266</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>46296</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3458,10 +3476,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$Q$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$R$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="15"/>
+                <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -3506,6 +3524,9 @@
                 </c:pt>
                 <c:pt idx="14">
                   <c:v>46266</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>46296</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3592,10 +3613,10 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$Q$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$R$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="15"/>
+                <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -3640,16 +3661,19 @@
                 </c:pt>
                 <c:pt idx="14">
                   <c:v>46266</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>46296</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$9:$Q$9</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$9:$R$9</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="15"/>
+                <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>532107.21</c:v>
                 </c:pt>
@@ -3694,6 +3718,9 @@
                 </c:pt>
                 <c:pt idx="14">
                   <c:v>90631.83</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>157869.14000000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5017,10 +5044,10 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="97"/>
-      <c r="B8" s="122" t="s">
+      <c r="B8" s="124" t="s">
         <v>101</v>
       </c>
-      <c r="C8" s="122"/>
+      <c r="C8" s="124"/>
       <c r="D8" s="103"/>
       <c r="E8" s="103"/>
       <c r="F8" s="103"/>
@@ -5502,15 +5529,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18.75" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="123" t="s">
+      <c r="A1" s="125" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="124"/>
-      <c r="C1" s="124"/>
-      <c r="D1" s="124"/>
-      <c r="E1" s="124"/>
-      <c r="F1" s="124"/>
-      <c r="G1" s="125"/>
+      <c r="B1" s="126"/>
+      <c r="C1" s="126"/>
+      <c r="D1" s="126"/>
+      <c r="E1" s="126"/>
+      <c r="F1" s="126"/>
+      <c r="G1" s="127"/>
     </row>
     <row r="2" spans="1:7" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -5611,22 +5638,22 @@
     </row>
     <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="8" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="126" t="s">
+      <c r="A8" s="128" t="s">
         <v>78</v>
       </c>
-      <c r="B8" s="127"/>
-      <c r="C8" s="128"/>
+      <c r="B8" s="129"/>
+      <c r="C8" s="130"/>
       <c r="D8" s="12"/>
       <c r="E8" s="12"/>
       <c r="F8" s="12"/>
       <c r="G8" s="12"/>
     </row>
     <row r="9" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="126" t="s">
+      <c r="A9" s="128" t="s">
         <v>112</v>
       </c>
-      <c r="B9" s="127"/>
-      <c r="C9" s="128"/>
+      <c r="B9" s="129"/>
+      <c r="C9" s="130"/>
       <c r="D9" s="13"/>
       <c r="E9" s="13"/>
     </row>
@@ -6294,10 +6321,10 @@
         <f>M5-I6</f>
         <v>511198.30999999994</v>
       </c>
-      <c r="O6" s="129" t="s">
+      <c r="O6" s="122" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="129"/>
+      <c r="P6" s="122"/>
       <c r="Q6" s="82">
         <f>(Q4/O4)-1</f>
         <v>-0.46666646370129106</v>
@@ -6428,11 +6455,11 @@
         <f>M8-I9</f>
         <v>484757.02999999991</v>
       </c>
-      <c r="O9" s="130" t="s">
+      <c r="O9" s="131" t="s">
         <v>87</v>
       </c>
-      <c r="P9" s="130"/>
-      <c r="Q9" s="130"/>
+      <c r="P9" s="131"/>
+      <c r="Q9" s="131"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="81" t="s">
@@ -6474,11 +6501,11 @@
         <f t="shared" ref="M10:M63" si="2">M9-I10</f>
         <v>475943.2699999999</v>
       </c>
-      <c r="O10" s="131" t="s">
+      <c r="O10" s="132" t="s">
         <v>88</v>
       </c>
-      <c r="P10" s="131"/>
-      <c r="Q10" s="131"/>
+      <c r="P10" s="132"/>
+      <c r="Q10" s="132"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="81" t="s">
@@ -6520,11 +6547,11 @@
         <f t="shared" si="2"/>
         <v>467129.50999999989</v>
       </c>
-      <c r="O11" s="132" t="s">
+      <c r="O11" s="133" t="s">
         <v>90</v>
       </c>
-      <c r="P11" s="132"/>
-      <c r="Q11" s="132"/>
+      <c r="P11" s="133"/>
+      <c r="Q11" s="133"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="83" t="s">
@@ -8334,10 +8361,10 @@
         <f>M5-I6</f>
         <v>1073254.2800000003</v>
       </c>
-      <c r="O6" s="129" t="s">
+      <c r="O6" s="122" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="129"/>
+      <c r="P6" s="122"/>
       <c r="Q6" s="82">
         <f>Q4/O4-1</f>
         <v>-0.36666658740617009</v>
@@ -8466,11 +8493,11 @@
         <f t="shared" si="2"/>
         <v>1017741.1400000004</v>
       </c>
-      <c r="O9" s="133" t="s">
+      <c r="O9" s="134" t="s">
         <v>86</v>
       </c>
-      <c r="P9" s="133"/>
-      <c r="Q9" s="133"/>
+      <c r="P9" s="134"/>
+      <c r="Q9" s="134"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="79" t="s">
@@ -8512,11 +8539,11 @@
         <f t="shared" si="2"/>
         <v>999236.76000000036</v>
       </c>
-      <c r="O10" s="130" t="s">
+      <c r="O10" s="131" t="s">
         <v>87</v>
       </c>
-      <c r="P10" s="130"/>
-      <c r="Q10" s="130"/>
+      <c r="P10" s="131"/>
+      <c r="Q10" s="131"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="79" t="s">
@@ -8558,11 +8585,11 @@
         <f t="shared" si="2"/>
         <v>980732.38000000035</v>
       </c>
-      <c r="O11" s="131" t="s">
+      <c r="O11" s="132" t="s">
         <v>88</v>
       </c>
-      <c r="P11" s="131"/>
-      <c r="Q11" s="131"/>
+      <c r="P11" s="132"/>
+      <c r="Q11" s="132"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="79" t="s">
@@ -11454,10 +11481,10 @@
         <f>M5-I6</f>
         <v>1727211.77</v>
       </c>
-      <c r="O6" s="129" t="s">
+      <c r="O6" s="122" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="129"/>
+      <c r="P6" s="122"/>
       <c r="Q6" s="82">
         <f>(Q4/O4)-1</f>
         <v>-0.26666663831011039</v>
@@ -11588,11 +11615,11 @@
         <f t="shared" ref="M9:M63" si="2">M8-I9</f>
         <v>1637873.24</v>
       </c>
-      <c r="O9" s="130" t="s">
+      <c r="O9" s="131" t="s">
         <v>87</v>
       </c>
-      <c r="P9" s="130"/>
-      <c r="Q9" s="130"/>
+      <c r="P9" s="131"/>
+      <c r="Q9" s="131"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="81" t="s">
@@ -11634,11 +11661,11 @@
         <f t="shared" si="2"/>
         <v>1608093.73</v>
       </c>
-      <c r="O10" s="131" t="s">
+      <c r="O10" s="132" t="s">
         <v>88</v>
       </c>
-      <c r="P10" s="131"/>
-      <c r="Q10" s="131"/>
+      <c r="P10" s="132"/>
+      <c r="Q10" s="132"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="81" t="s">
@@ -11680,11 +11707,11 @@
         <f t="shared" si="2"/>
         <v>1578314.22</v>
       </c>
-      <c r="O11" s="132" t="s">
+      <c r="O11" s="133" t="s">
         <v>90</v>
       </c>
-      <c r="P11" s="132"/>
-      <c r="Q11" s="132"/>
+      <c r="P11" s="133"/>
+      <c r="Q11" s="133"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="81" t="s">
@@ -13460,10 +13487,10 @@
         <f>M5-I6</f>
         <v>88254.450000000012</v>
       </c>
-      <c r="O6" s="129" t="s">
+      <c r="O6" s="122" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="129"/>
+      <c r="P6" s="122"/>
       <c r="Q6" s="82">
         <f>(Q4/O4)-1</f>
         <v>-0.14999919494129588</v>
@@ -13549,11 +13576,11 @@
         <f t="shared" ref="M9:M63" si="2">M8-I9</f>
         <v>83689.590000000026</v>
       </c>
-      <c r="O9" s="130" t="s">
+      <c r="O9" s="131" t="s">
         <v>87</v>
       </c>
-      <c r="P9" s="130"/>
-      <c r="Q9" s="130"/>
+      <c r="P9" s="131"/>
+      <c r="Q9" s="131"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="39"/>
@@ -13580,11 +13607,11 @@
         <f t="shared" si="2"/>
         <v>82167.97000000003</v>
       </c>
-      <c r="O10" s="131" t="s">
+      <c r="O10" s="132" t="s">
         <v>88</v>
       </c>
-      <c r="P10" s="131"/>
-      <c r="Q10" s="131"/>
+      <c r="P10" s="132"/>
+      <c r="Q10" s="132"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="39"/>
@@ -13611,11 +13638,11 @@
         <f t="shared" si="2"/>
         <v>80646.350000000035</v>
       </c>
-      <c r="O11" s="132" t="s">
+      <c r="O11" s="133" t="s">
         <v>90</v>
       </c>
-      <c r="P11" s="132"/>
-      <c r="Q11" s="132"/>
+      <c r="P11" s="133"/>
+      <c r="Q11" s="133"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="39"/>
@@ -15298,10 +15325,10 @@
       <c r="N6" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="P6" s="129" t="s">
+      <c r="P6" s="122" t="s">
         <v>89</v>
       </c>
-      <c r="Q6" s="129"/>
+      <c r="Q6" s="122"/>
       <c r="R6" s="82">
         <f>(R4/P4)-1</f>
         <v>-1</v>
@@ -15400,9 +15427,9 @@
       <c r="N9" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="P9" s="134"/>
-      <c r="Q9" s="134"/>
-      <c r="R9" s="134"/>
+      <c r="P9" s="123"/>
+      <c r="Q9" s="123"/>
+      <c r="R9" s="123"/>
     </row>
     <row r="10" spans="2:19" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="39"/>
@@ -15432,9 +15459,9 @@
       <c r="N10" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="P10" s="134"/>
-      <c r="Q10" s="134"/>
-      <c r="R10" s="134"/>
+      <c r="P10" s="123"/>
+      <c r="Q10" s="123"/>
+      <c r="R10" s="123"/>
     </row>
     <row r="11" spans="2:19" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="39"/>
@@ -15464,9 +15491,9 @@
       <c r="N11" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="P11" s="134"/>
-      <c r="Q11" s="134"/>
-      <c r="R11" s="134"/>
+      <c r="P11" s="123"/>
+      <c r="Q11" s="123"/>
+      <c r="R11" s="123"/>
     </row>
     <row r="12" spans="2:19" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="39"/>
@@ -17634,14 +17661,14 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{420301BD-1EC9-404C-9D58-1869DDAA2327}">
-  <dimension ref="B2:Q9"/>
+  <dimension ref="B2:R9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="17" width="13.33203125" customWidth="1"/>
+    <col min="3" max="18" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:18" x14ac:dyDescent="0.3">
       <c r="C2" s="85">
         <v>45839</v>
       </c>
@@ -17687,8 +17714,11 @@
       <c r="Q2" s="85">
         <v>46266</v>
       </c>
-    </row>
-    <row r="3" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="R2" s="85">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="3" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B3" s="84" t="s">
         <v>95</v>
       </c>
@@ -17741,8 +17771,12 @@
       <c r="Q3" s="27">
         <v>3796974.4</v>
       </c>
-    </row>
-    <row r="4" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="R3" s="27">
+        <f>3713217.08</f>
+        <v>3713217.08</v>
+      </c>
+    </row>
+    <row r="4" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B4" s="84" t="s">
         <v>96</v>
       </c>
@@ -17791,8 +17825,11 @@
       <c r="Q4" s="27">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="R4" s="27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B5" s="84" t="s">
         <v>76</v>
       </c>
@@ -17841,8 +17878,11 @@
         <f>16179.2</f>
         <v>16179.2</v>
       </c>
-    </row>
-    <row r="6" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="R5" s="27">
+        <v>28180.61</v>
+      </c>
+    </row>
+    <row r="6" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B6" s="84" t="s">
         <v>77</v>
       </c>
@@ -17893,8 +17933,11 @@
         <f>74452.63</f>
         <v>74452.63</v>
       </c>
-    </row>
-    <row r="7" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="R6" s="27">
+        <v>129688.53</v>
+      </c>
+    </row>
+    <row r="7" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B7" s="84" t="s">
         <v>97</v>
       </c>
@@ -17929,8 +17972,9 @@
       <c r="O7" s="27"/>
       <c r="P7" s="27"/>
       <c r="Q7" s="27"/>
-    </row>
-    <row r="8" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="R7" s="27"/>
+    </row>
+    <row r="8" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B8" s="84" t="s">
         <v>8</v>
       </c>
@@ -17964,8 +18008,9 @@
       <c r="O8" s="27"/>
       <c r="P8" s="27"/>
       <c r="Q8" s="27"/>
-    </row>
-    <row r="9" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="R8" s="27"/>
+    </row>
+    <row r="9" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B9" s="84" t="s">
         <v>99</v>
       </c>
@@ -18028,6 +18073,10 @@
       <c r="Q9" s="96">
         <f t="shared" si="2"/>
         <v>90631.83</v>
+      </c>
+      <c r="R9" s="96">
+        <f t="shared" ref="R9" si="3">SUM(R4:R8)</f>
+        <v>157869.14000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>